<commit_message>
docs(cadrage v4): §24.8 resilience integrale (856 runs)
- §24.8.1 distributions (P50/P75/P95/P99, ratios queue lourde)
- §24.8.2 gradient d'intensite (courbe plate documentee honnetement)
- §24.8.3 cascade 1-5 pannes (sensibilite 5x plus faible pour EVENT)
- §24.8.4 verdict + 5 limites explicites (in-silico, pas IEC 60050)
- DOCX regenere avec 3 PNG resilience embarques
- XLSX enrichi d'une feuille Resilience_856_runs (P95/P99, gradient,
  cascade, MTTR, sensibilite)

Resultats : EVENT a la meilleure queue (P95 220k vs 261k OF),
5x moins sensible a la cascade (+4.5% vs +23.2%), MTTR 1.6-2x
plus court. Gradient d'intensite plat -> protocole revisable.
</commit_message>
<xml_diff>
--- a/docs/cadrage_v4_kpis.xlsx
+++ b/docs/cadrage_v4_kpis.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="XL_4000_runs" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Random_1600_runs" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decomposition_2x2" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resilience_856_runs" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -55,6 +56,9 @@
       <color rgb="002CA02C"/>
       <sz val="12"/>
     </font>
+    <font>
+      <i val="1"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -86,7 +90,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -100,6 +104,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1865,4 +1870,855 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I41"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>§24.8 — Analyse de résilience (856 runs : 256 distrib + 300 gradient + 300 cascade)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>§24.8.1 — Distributions de coût (256 runs)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Doctrine</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Moyenne</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>σ</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>P50</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>P75</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>P95</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>P99</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Max</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>OF</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>64</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>152 028 €</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>55 230 €</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>136 213 €</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>174 280 €</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>261 855 €</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>316 851 €</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>359 912 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>64</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>126 940 €</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>49 975 €</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>119 951 €</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>147 237 €</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>222 570 €</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>289 395 €</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>321 560 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>OF+EVENT</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>64</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>146 672 €</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>56 155 €</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>135 383 €</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>167 709 €</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>276 428 €</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>310 432 €</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>342 564 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>EVENT</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>64</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>121 866 €</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>50 233 €</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>112 829 €</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>141 320 €</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>220 793 €</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>286 827 €</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>314 621 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="9"/>
+    <row r="10"/>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>§24.8.2 — Gradient d'intensité (300 runs) — coût moyen €</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Intensité</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>OF</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>OF+EVENT</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>EVENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>x0.5</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>114 049 €</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>101 007 €</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>113 191 €</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>100 566 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>x1.0</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>117 336 €</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>98 364 €</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>113 029 €</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>97 655 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>x1.5</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>119 776 €</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>99 664 €</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>113 464 €</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>99 437 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>x2.0</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>117 605 €</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>99 990 €</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>113 980 €</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>100 594 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>x2.5</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>114 925 €</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>100 969 €</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>113 484 €</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>99 499 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="18"/>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>Note : courbe plate → ces variations d'intensité ne discriminent pas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20"/>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>§24.8.3 — Cascade de pannes simultanées (300 runs) — coût moyen €</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Pannes simultanées</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>OF</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>OF+EVENT</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>EVENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>107 116 €</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>68 524 €</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>101 392 €</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>67 198 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>112 506 €</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>72 831 €</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>103 452 €</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>68 398 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>120 826 €</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>75 345 €</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>105 518 €</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>69 145 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>127 923 €</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>78 276 €</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>107 685 €</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>70 087 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>131 954 €</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>80 370 €</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>110 331 €</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>70 247 €</t>
+        </is>
+      </c>
+    </row>
+    <row r="28"/>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Time-to-recover (jours)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Pannes simultanées</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>OF</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>OF+EVENT</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>EVENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>5.8 j</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>3.0 j</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>5.7 j</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>2.9 j</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>5.9 j</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>3.5 j</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>5.7 j</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>3.0 j</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>5.9 j</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>3.9 j</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>5.7 j</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>3.1 j</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>5.7 j</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>4.9 j</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>5.7 j</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>3.5 j</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>5.5 j</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>5.1 j</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>5.7 j</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>3.5 j</t>
+        </is>
+      </c>
+    </row>
+    <row r="36"/>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Sensibilité au choc — Δ relatif 1→5 pannes</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="7" t="inlineStr">
+        <is>
+          <t>OF</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>+23.2 %</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="7" t="inlineStr">
+        <is>
+          <t>FLUX</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>+17.3 %</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="7" t="inlineStr">
+        <is>
+          <t>OF+EVENT</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>+8.8 %</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>EVENT</t>
+        </is>
+      </c>
+      <c r="B41" s="8" t="inlineStr">
+        <is>
+          <t>+4.5 %</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A29:I29"/>
+    <mergeCell ref="A19:I19"/>
+    <mergeCell ref="A11:I11"/>
+    <mergeCell ref="A37:I37"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A3:I3"/>
+    <mergeCell ref="A21:I21"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>